<commit_message>
Nuevo incidente agregado - caída al mismo nivel
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M205"/>
+  <dimension ref="A1:M206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10532,6 +10532,65 @@
       </c>
       <c r="L205" t="inlineStr"/>
       <c r="M205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>caída al mismo nivel</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="n">
+        <v>46041</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Agente de carga</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Agente de carga</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Caidas a nivel</t>
+        </is>
+      </c>
+      <c r="G206" t="n">
+        <v>1</v>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Pasa una vez o más al año</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Se les notifica que siendo a las 06:45 personal de Menzies estaban retirando carga de los cuartos fríos al momento de movilizar una posición en el pasillo el señor Brayan Ezequiel Coguaix Martinez con gafete 26-00415 se tropieza y cae en los rodos indicando que no se puede movilizar, se procede a informarle a alfa 10 de lo sucedido se hace presente Ray Varga el brigadista de COMBEX-IM con el gafete 25-E0208 para atenderlo se traslada a la persona enfrente de la basculas 3 Ray Vargas procede a la revisión indica que es una herida expuesta se le informa a Carlos García para coordinar a los bomberos.</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante x Pasa una vez o más al año</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nuevo incidente agregado - 2955108970108
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -22,16 +22,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -431,71 +419,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M207"/>
+  <dimension ref="A1:M208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Área</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Puesto</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Causa</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Días_Perdidos</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Severidad</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Probabilidad</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Riesgo</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Hora del Evento</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Riesgo_valor</t>
         </is>
@@ -507,7 +495,7 @@
           <t>caída al mismo nivel</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="1" t="n">
         <v>46041</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -3638,7 +3626,7 @@
           <t xml:space="preserve">Caída a distinto nivel </t>
         </is>
       </c>
-      <c r="B207" s="2" t="n">
+      <c r="B207" s="1" t="n">
         <v>46079</v>
       </c>
       <c r="C207" t="inlineStr">
@@ -3690,6 +3678,65 @@
         </is>
       </c>
       <c r="M207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2955108970108</t>
+        </is>
+      </c>
+      <c r="B208" s="1" t="n">
+        <v>46128</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conserje </t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conserje </t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Casi Accidente</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Caída de producto de limpieza en ambos ojos</t>
+        </is>
+      </c>
+      <c r="G208" t="n">
+        <v>2</v>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Lesión leve o sin impacto</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Pasa una vez o más al año</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>EL día jueves el colaborador Lester alexander Chua , realizando sus labores y manipulando una pasta de limpieza de inodoros le cayo en los ojos donde se, activo el protocolo y se le refirió al IGSS inmediatamente.</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Lesión leve o sin impacto x Pasa una vez o más al año</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>11:26</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3706,77 +3753,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID_Riesgo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Clasificación de peligro</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Peligro</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Fuente o actividad</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Tipo de puesto</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Probabilidad</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unnamed: 6</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Severidad</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Unnamed: 8</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Nivel de Riesgo</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Unnamed: 10</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Jerarquía de riesgo</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Medidas de control</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Hallazgos/Oportunidades de mejora</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Nivel</t>
         </is>
@@ -6281,17 +6328,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Capacitaciones</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Asistentes</t>
         </is>

</xml_diff>

<commit_message>
Nuevo incidente agregado - 26-02241
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M208"/>
+  <dimension ref="A1:M209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3737,6 +3737,65 @@
         </is>
       </c>
       <c r="M208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>26-02241</t>
+        </is>
+      </c>
+      <c r="B209" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Oficial de rampa</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Oficial de rampa</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Caidas a diferente nivel</t>
+        </is>
+      </c>
+      <c r="G209" t="n">
+        <v>2</v>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Lesión Severa</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Pasa una vez o más al año</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>El día de ayer el colaborador Ean Karlo Arriaga de la empresa DHL sufrió una caída en el cuarto frio numero 5, por lo que se le dio los primero  auxilios, y se procedió a llamar a los servicios de emergencia para el traslado del joven.</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Lesión Severa x Pasa una vez o más al año</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nuevo incidente agregado - 26-00110
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M209"/>
+  <dimension ref="A1:M210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3796,6 +3796,66 @@
         </is>
       </c>
       <c r="M209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>26-00110</t>
+        </is>
+      </c>
+      <c r="B210" s="1" t="n">
+        <v>46193</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supervisor de aduanas </t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supervisor de aduanas </t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Incidente</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Presión baja y glucosa alta</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>0</v>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Lesión leve o sin impacto</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Podría pasar</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Se brindo asistencia a colaboradora de SAT. 
+En coordinación con bomberos y alerta médica por traslado a un centro médico.</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Lesión leve o sin impacto x Podría pasar</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nuevo incidente agregado - E0942
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M210"/>
+  <dimension ref="A1:M211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3856,6 +3856,65 @@
         </is>
       </c>
       <c r="M210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>E0942</t>
+        </is>
+      </c>
+      <c r="B211" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Jefe de grupo</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Jefe de grupo</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Caidas a diferente nivel</t>
+        </is>
+      </c>
+      <c r="G211" t="n">
+        <v>30</v>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Lesión Severa</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Pasó alguna vez</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>El día 3 de agosto del año 2026 el colaborador Walter Tobar tubo un accidente, en el  que se fracturo  la cadera debido  a que la caida fue a deferente nivel.</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Lesión Severa x Pasó alguna vez</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>7:30</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nuevo incidente agregado - 0515
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M211"/>
+  <dimension ref="A1:M212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3915,6 +3915,65 @@
         </is>
       </c>
       <c r="M211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>0515</t>
+        </is>
+      </c>
+      <c r="B212" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Operador de montacargas</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Operador de montacargas</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Casi Accidente</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Contusiones leves y severas (caida de objetos)</t>
+        </is>
+      </c>
+      <c r="G212" t="n">
+        <v>12</v>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Podría pasar</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Colaborador lastimado por objeto proyectado hacia el rostro, impactando labio superior ocasionando una contusión  y herida, que requirió el traslado del colaborador a un centro asistencial. </t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante x Podría pasar</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nuevo incidente agregado - 26-0001183
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M212"/>
+  <dimension ref="A1:M213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3974,6 +3974,65 @@
         </is>
       </c>
       <c r="M212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>26-0001183</t>
+        </is>
+      </c>
+      <c r="B213" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Café internet</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Café internet</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Casi Accidente</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Caidas a diferente nivel</t>
+        </is>
+      </c>
+      <c r="G213" t="n">
+        <v>0</v>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Podría pasar</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>La clienta se sentó en una silla que no soporto su el peso y se abrió, provocando la caída del cliente , y provoco que se lastimara el brazo derecho</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante x Podría pasar</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>13.05</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nuevo incidente agregado - 25-E0433
</commit_message>
<xml_diff>
--- a/SSO_datos_ejemplo.xlsx
+++ b/SSO_datos_ejemplo.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M213"/>
+  <dimension ref="A1:M214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4033,6 +4033,65 @@
         </is>
       </c>
       <c r="M213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>25-E0433</t>
+        </is>
+      </c>
+      <c r="B214" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Receptor de carga</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Receptor de carga</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Incidente</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Caidas a nivel</t>
+        </is>
+      </c>
+      <c r="G214" t="n">
+        <v>9</v>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Pasó alguna vez</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>El colaborador se enredo con un fleje suelto, el cual provoco la caída y a raíz de eso el colaborador se lastimo la oreja izquierda, por lo que se tuvo que coordinar la llegada de los bomberos de SSEI   y luego el traslado del colaborador al IGSS de accidentes.</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Lesión incapacitante x Pasó alguna vez</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>9:22</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>